<commit_message>
Document LTRP general rule: max 6 plans, each January sums 1/6 each.
Example: 2026 grant of 70,000 pays in Jan 2027 as 1/6 of 2026 plus 1/6 of 2025–2022.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LTRP/LTRP.xlsx
+++ b/LTRP/LTRP.xlsx
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +48,10 @@
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="001F4E79"/>
     </font>
   </fonts>
   <fills count="5">
@@ -99,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -129,6 +133,7 @@
     <xf numFmtId="4" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -495,11 +500,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -535,167 +540,169 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Moneda</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Fórmula del cobro 31/01</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>SUMAR (Valor nominal ÷ 6) de cada plan vigente desde 2022</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>REGLA GENERAL</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Se acumulan como máximo 6 planes; cada enero se suma el 1/6 de cada uno</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Ejemplo plan 2026</t>
+          <t>Ejemplo — otorgado 70.000 en 2026</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>70.000 ÷ 6 = 11.666,67  +  1/6 de LTRP 2022…2025</t>
+          <t>Ene 2027 = 1/6·2026 + 1/6·2025 + 1/6·2024 + 1/6·2023 + 1/6·2022</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Duración por plan</t>
+          <t>Ventana</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>6 cobros anuales (1/6 por año) en 31/01</t>
+          <t>Cuando entra un plan nuevo, el que ya cobró 6 veces sale de la suma</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>Fecha de cada cobro</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>31/01</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>Composición del pago</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>50% fijo + 50% variable (acción MELI)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Pago base 31/01/2027 = suma de cinco 1/6</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>32803.67</v>
-      </c>
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · LTRP 2022 ÷ 6</t>
+          <t>Pago base ene-2027 (suma de 1/6)</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>5000</v>
+        <v>32803.67</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · LTRP 2023 ÷ 6</t>
+          <t xml:space="preserve">  · 1/6 LTRP 2026 (70.000÷6)</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>5000</v>
+        <v>11666.6666666667</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · LTRP 2024 ÷ 6</t>
+          <t xml:space="preserve">  · 1/6 LTRP 2025 (36.822÷6)</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>5000</v>
+        <v>6137</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · LTRP 2025 ÷ 6</t>
+          <t xml:space="preserve">  · 1/6 LTRP 2024 (30.000÷6)</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>6137</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · LTRP 2026 ÷ 6</t>
+          <t xml:space="preserve">  · 1/6 LTRP 2023 (30.000÷6)</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>11666.6666666667</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Estimación portal MELI 2027</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>35332</v>
+          <t xml:space="preserve">  · 1/6 LTRP 2022 (30.000÷6)</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>5000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>Estimación portal MELI 2027</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>35332</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>Factor MELI implícito (solo variable)</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B18" s="3" t="n">
         <v>1.1542</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="6" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Total valor nominal planes vigentes</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>196822</v>
-      </c>
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Planes vigentes</t>
+          <t>Planes vigentes hoy</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
@@ -703,18 +710,38 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr"/>
-      <c r="B21" s="3" t="inlineStr"/>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Tope de planes por cobro</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
+          <t>Total valor nominal planes vigentes</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>196822</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>El valor nominal (ej. 70.000) es el plan asignado ese año, NO el cobro anual. El cobro = suma de los ÷6 activos. El 50% variable mueve el total vs la base. Ingreso por bono; no es gasto CIUDAD/SOL.</t>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>70.000 es el plan OTORGADO en 2026, no el cobro. El cobro de enero = suma de hasta 6 tramos de Nominal÷6. Ingreso por bono; no es gasto CIUDAD/SOL.</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1833,7 @@
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>Suma 1/6 de LTRP 2022..2026 = 5000+5000+5000+6137+11666.67 · portal 35.332</t>
+          <t>Regla: máx 6 planes · ene-2027 = 1/6·2026+2025+2024+2023+2022 · portal 35.332</t>
         </is>
       </c>
     </row>
@@ -1974,8 +2001,8 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="65" customWidth="1" min="1" max="1"/>
-    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
@@ -1986,11 +2013,17 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Pago 31/01/2027 = suma de (Nominal ÷ 6) de cada plan desde 2022</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>Pago ene-2027 = 1/6·2026 + 1/6·2025 + 1/6·2024 + 1/6·2023 + 1/6·2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Regla: máximo 6 planes acumulados; cada enero se suma el 1/6 de cada uno</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1999,12 +2032,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Valor nominal USD</t>
+          <t>Valor otorgado USD</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Nominal ÷ 6</t>
+          <t>1/6 en este pago</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2031,51 +2064,51 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>LTRP 2022</t>
+          <t>LTRP 2026</t>
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>30000</v>
+        <v>70000</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>5000</v>
+        <v>11666.66666666667</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>2500</v>
+        <v>5833.333333333333</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>2500</v>
+        <v>5833.333333333333</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>2885.5</v>
+        <v>6732.833333333332</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>5385.5</v>
+        <v>12566.16666666666</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>LTRP 2023</t>
+          <t>LTRP 2025</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>30000</v>
+        <v>36822</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>5000</v>
+        <v>6137</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2500</v>
+        <v>3068.5</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>2500</v>
+        <v>3068.5</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>2885.5</v>
+        <v>3541.6627</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>5385.5</v>
+        <v>6610.1627</v>
       </c>
     </row>
     <row r="6">
@@ -2106,57 +2139,57 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>LTRP 2025</t>
+          <t>LTRP 2023</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>36822</v>
+        <v>30000</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>6137</v>
+        <v>5000</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>3068.5</v>
+        <v>2500</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>3068.5</v>
+        <v>2500</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>3541.6627</v>
+        <v>2885.5</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>6610.1627</v>
+        <v>5385.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>LTRP 2026</t>
+          <t>LTRP 2022</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>11666.66666666667</v>
+        <v>5000</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>5833.333333333333</v>
+        <v>2500</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>5833.333333333333</v>
+        <v>2500</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>6732.833333333332</v>
+        <v>2885.5</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>12566.16666666666</v>
+        <v>5385.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>SUMA (pago base 31/01/2027)</t>
+          <t>SUMA (pago base ene-2027)</t>
         </is>
       </c>
       <c r="B9" s="8">
@@ -2193,14 +2226,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pago base = 30000/6 + 30000/6 + 30000/6 + 36822/6 + 70000/6</t>
+          <t>1/6·70000 + 1/6·36822 + 1/6·30000 + 1/6·30000 + 1/6·30000</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
       <c r="B12">
-        <f> 5.000 + 5.000 + 5.000 + 6.137 + 11.666,67 = 32.803,67</f>
+        <f> 11.666,67 + 6.137 + 5.000 + 5.000 + 5.000 = 32.803,67</f>
         <v/>
       </c>
     </row>
@@ -2210,7 +2243,7 @@
           <t>Estimación portal MELI (agosto 2026)</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n">
+      <c r="B13" s="18" t="n">
         <v>35332</v>
       </c>
     </row>
@@ -2239,12 +2272,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Pago final</t>
+          <t>Tope</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>(suma ÷6)×50% fijo + (suma ÷6)×50%×factor_MELI</t>
+          <t>Nunca más de 6 planes en un mismo enero; el más viejo sale al completar 6 cobros</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Note that LTRP base vs portal estimate gap is MELI stock price.
Document 32,803.67 base vs 35,332 estimate (+2,528.33) as the variable 50% adjusted by share value.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LTRP/LTRP.xlsx
+++ b/LTRP/LTRP.xlsx
@@ -500,10 +500,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="1" max="1"/>
     <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -676,72 +676,94 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Estimación portal MELI 2027</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="5" t="n">
         <v>35332</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Factor MELI implícito (solo variable)</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="n">
-        <v>1.1542</v>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Diferencia (base → estimado)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>2528.33</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr"/>
-      <c r="B19" s="3" t="inlineStr"/>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Motivo de la diferencia</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Valor de la acción MELI sobre el 50% variable (el 50% fijo no cambia)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Planes vigentes hoy</t>
+          <t>Factor acción implícito (solo variable)</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>5</v>
+        <v>1.1542</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Tope de planes por cobro</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n">
-        <v>6</v>
-      </c>
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Total valor nominal planes vigentes</t>
+          <t>Planes vigentes hoy</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>196822</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr"/>
-      <c r="B23" s="3" t="inlineStr"/>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Tope de planes por cobro</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t>Total valor nominal planes vigentes</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>196822</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>70.000 es el plan OTORGADO en 2026, no el cobro. El cobro de enero = suma de hasta 6 tramos de Nominal÷6. Ingreso por bono; no es gasto CIUDAD/SOL.</t>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>70.000 es el plan OTORGADO en 2026, no el cobro. Base 32.803,67 = suma de 1/6. Estimado 35.332 = misma suma ajustada por el precio de la acción MELI en la mitad variable. Ingreso por bono; no es gasto CIUDAD/SOL.</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1855,7 @@
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>Regla: máx 6 planes · ene-2027 = 1/6·2026+2025+2024+2023+2022 · portal 35.332</t>
+          <t>Base 32803.67 vs estimado 35332: diferencia por valor de la acción MELI (50% variable)</t>
         </is>
       </c>
     </row>
@@ -1998,7 +2020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -2250,32 +2272,54 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Factor MELI usado en esta hoja (implícito)</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1.1542</v>
+          <t>Diferencia vs base</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="n">
+        <v>2528.330000000002</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>*Variable estimado</t>
+          <t>Motivo diferencia</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Variable base × factor MELI implícito (35.332 vs base 32.803,67)</t>
+          <t>Valor de la acción MELI (ajusta solo el 50% variable; el fijo no cambia)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Factor acción implícito (solo variable)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.1542</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>*Variable estimado</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Variable base × factor de la acción (35.332 − 32.803,67 = efecto MELI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Tope</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Nunca más de 6 planes en un mismo enero; el más viejo sale al completar 6 cobros</t>
         </is>

</xml_diff>

<commit_message>
Note LTRP 2026 grant is fully collected only in 2032.
Document that the 70,000 plan pays six January tranches (2027–2032) and the last 1/6 completes the grant in 2032.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LTRP/LTRP.xlsx
+++ b/LTRP/LTRP.xlsx
@@ -120,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -155,6 +155,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -536,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -588,8 +589,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr"/>
-      <c r="B5" s="4" t="inlineStr"/>
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -604,160 +605,172 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Ejemplo</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Otorgado 70.000 en 2026 → ene-2027 = 1/6·2026 + 1/6·2025 + 1/6·2024 + 1/6·2023 + 1/6·2022</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Plan 2026 completo</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Recién en 2032 se cobra el 6/6 y se completa la totalidad del plan otorgado en 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Fórmula con acción</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>(N/6)×50% fijo + (N/6)×50% × (P_año / P_otorgamiento)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Total estimado a cobrar 2027</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B11" s="5" t="n">
         <v>35332</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Total estimado a cobrar 2028</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>36847</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Total estimado a cobrar 2029</t>
+          <t>Total estimado a cobrar 2028</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>32284</v>
+        <v>36847</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Total estimado a cobrar 2030</t>
+          <t>Total estimado a cobrar 2029</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>25001</v>
+        <v>32284</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>Total estimado a cobrar 2030</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>25001</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>Total estimado a cobrar 2031</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B15" s="6" t="n">
         <v>19379</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Total estimado a cobrar 2032</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B16" s="5" t="n">
         <v>13056</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Total acumulado pendiente de pago</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B17" s="5" t="n">
         <v>161899</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr"/>
-      <c r="B17" s="7" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Base 2027 sin efecto acción (suma 1/6)</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>32803.67</v>
-      </c>
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Diferencia 2027 por valor de la acción</t>
+          <t>Base 2027 sin efecto acción (suma 1/6)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>2528.33</v>
+        <v>32803.67</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>Diferencia 2027 por valor de la acción</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>2528.33</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>Precio acción estimado 2027</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B21" s="7" t="n">
         <v>1765.02</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr"/>
-      <c r="B21" s="3" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Metodología precio</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Año 1: promedio 60 días + 3% cierre 2026 · Luego +8% anual</t>
-        </is>
-      </c>
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
+          <t>Metodología precio</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Año 1: promedio 60 días + 3% cierre 2026 · Luego +8% anual</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Ingreso por bono MELI; independiente de CIUDAD / SOL / propiedades.</t>
         </is>
@@ -774,7 +787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1079,7 +1092,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1">
+    <row r="19" ht="48" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Regla general</t>
@@ -1087,12 +1100,25 @@
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>Máximo 6 planes. Cada enero se suma el 1/6 de cada plan activo. Ej.: otorgado 70.000 en 2026 → ene-2027 = 1/6·2026 + 1/6·2025 + … + 1/6·2022, cada tramo ajustado 50/50 por la acción.</t>
+          <t>Máximo 6 planes. Cada enero se suma el 1/6 de cada plan activo. Ej.: otorgado 70.000 en 2026 → ene-2027 = 1/6·2026 + 1/6·2025 + … + 1/6·2022, cada tramo ajustado 50/50 por la acción. Recién en 2032 se cobra el 6/6 y se completa la totalidad del plan 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Plan LTRP 2026 (70.000)</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>6 cobros ene-2027…ene-2032 · la totalidad del plan se completa recién en 2032 (último 1/6 = 13.056)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="B21:I21"/>
     <mergeCell ref="B19:I19"/>
     <mergeCell ref="A13:I13"/>
   </mergeCells>
@@ -1338,31 +1364,31 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Cobros ene-2027 a ene-2032 · otorgado 70000</t>
+          <t>6 cobros ene-2027…ene-2032 · recién en 2032 se completa la totalidad del plan otorgado en 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
       <c r="B7" s="3" t="n"/>
-      <c r="C7" s="21">
+      <c r="C7" s="22">
         <f>SUM(C2:C6)</f>
         <v/>
       </c>
       <c r="D7" s="7" t="n"/>
-      <c r="E7" s="22">
+      <c r="E7" s="23">
         <f>SUM(E2:E6)</f>
         <v/>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="23">
         <f>SUM(F2:F6)</f>
         <v/>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="23">
         <f>SUM(G2:G6)</f>
         <v/>
       </c>
@@ -1409,7 +1435,7 @@
       <c r="A2" s="3" t="n">
         <v>2027</v>
       </c>
-      <c r="B2" s="23" t="n">
+      <c r="B2" s="24" t="n">
         <v>1765.02</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -1422,7 +1448,7 @@
       <c r="A3" s="3" t="n">
         <v>2028</v>
       </c>
-      <c r="B3" s="23" t="n">
+      <c r="B3" s="24" t="n">
         <v>1906.22</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1435,7 +1461,7 @@
       <c r="A4" s="3" t="n">
         <v>2029</v>
       </c>
-      <c r="B4" s="23" t="n">
+      <c r="B4" s="24" t="n">
         <v>2058.72</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1448,7 +1474,7 @@
       <c r="A5" s="3" t="n">
         <v>2030</v>
       </c>
-      <c r="B5" s="23" t="n">
+      <c r="B5" s="24" t="n">
         <v>2223.42</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1461,7 +1487,7 @@
       <c r="A6" s="3" t="n">
         <v>2031</v>
       </c>
-      <c r="B6" s="23" t="n">
+      <c r="B6" s="24" t="n">
         <v>2401.29</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1474,7 +1500,7 @@
       <c r="A7" s="3" t="n">
         <v>2032</v>
       </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="24" t="n">
         <v>2593.39</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1556,301 +1582,301 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>Plan</t>
         </is>
       </c>
-      <c r="B1" s="24" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>31/01/2023</t>
         </is>
       </c>
-      <c r="C1" s="24" t="inlineStr">
+      <c r="C1" s="25" t="inlineStr">
         <is>
           <t>31/01/2024</t>
         </is>
       </c>
-      <c r="D1" s="24" t="inlineStr">
+      <c r="D1" s="25" t="inlineStr">
         <is>
           <t>31/01/2025</t>
         </is>
       </c>
-      <c r="E1" s="24" t="inlineStr">
+      <c r="E1" s="25" t="inlineStr">
         <is>
           <t>31/01/2026</t>
         </is>
       </c>
-      <c r="F1" s="24" t="inlineStr">
+      <c r="F1" s="25" t="inlineStr">
         <is>
           <t>31/01/2027</t>
         </is>
       </c>
-      <c r="G1" s="24" t="inlineStr">
+      <c r="G1" s="25" t="inlineStr">
         <is>
           <t>31/01/2028</t>
         </is>
       </c>
-      <c r="H1" s="24" t="inlineStr">
+      <c r="H1" s="25" t="inlineStr">
         <is>
           <t>31/01/2029</t>
         </is>
       </c>
-      <c r="I1" s="24" t="inlineStr">
+      <c r="I1" s="25" t="inlineStr">
         <is>
           <t>31/01/2030</t>
         </is>
       </c>
-      <c r="J1" s="24" t="inlineStr">
+      <c r="J1" s="25" t="inlineStr">
         <is>
           <t>31/01/2031</t>
         </is>
       </c>
-      <c r="K1" s="24" t="inlineStr">
+      <c r="K1" s="25" t="inlineStr">
         <is>
           <t>31/01/2032</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>LTRP 2022</t>
         </is>
       </c>
-      <c r="B2" s="25" t="inlineStr">
+      <c r="B2" s="26" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="C2" s="25" t="inlineStr">
+      <c r="C2" s="26" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="D2" s="25" t="inlineStr">
+      <c r="D2" s="26" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="E2" s="25" t="inlineStr">
+      <c r="E2" s="26" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="F2" s="25" t="inlineStr">
+      <c r="F2" s="26" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="G2" s="25" t="inlineStr">
+      <c r="G2" s="26" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="H2" s="25" t="inlineStr"/>
-      <c r="I2" s="25" t="inlineStr"/>
-      <c r="J2" s="25" t="inlineStr"/>
-      <c r="K2" s="25" t="inlineStr"/>
+      <c r="H2" s="26" t="inlineStr"/>
+      <c r="I2" s="26" t="inlineStr"/>
+      <c r="J2" s="26" t="inlineStr"/>
+      <c r="K2" s="26" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>LTRP 2023</t>
         </is>
       </c>
-      <c r="B3" s="25" t="inlineStr"/>
-      <c r="C3" s="25" t="inlineStr">
+      <c r="B3" s="26" t="inlineStr"/>
+      <c r="C3" s="26" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="D3" s="25" t="inlineStr">
+      <c r="D3" s="26" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="E3" s="25" t="inlineStr">
+      <c r="E3" s="26" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="F3" s="25" t="inlineStr">
+      <c r="F3" s="26" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="G3" s="25" t="inlineStr">
+      <c r="G3" s="26" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="H3" s="25" t="inlineStr">
+      <c r="H3" s="26" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="I3" s="25" t="inlineStr"/>
-      <c r="J3" s="25" t="inlineStr"/>
-      <c r="K3" s="25" t="inlineStr"/>
+      <c r="I3" s="26" t="inlineStr"/>
+      <c r="J3" s="26" t="inlineStr"/>
+      <c r="K3" s="26" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>LTRP 2024</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr"/>
-      <c r="C4" s="25" t="inlineStr"/>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="B4" s="26" t="inlineStr"/>
+      <c r="C4" s="26" t="inlineStr"/>
+      <c r="D4" s="26" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="E4" s="25" t="inlineStr">
+      <c r="E4" s="26" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="F4" s="25" t="inlineStr">
+      <c r="F4" s="26" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="G4" s="25" t="inlineStr">
+      <c r="G4" s="26" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="H4" s="25" t="inlineStr">
+      <c r="H4" s="26" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="I4" s="25" t="inlineStr">
+      <c r="I4" s="26" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="J4" s="25" t="inlineStr"/>
-      <c r="K4" s="25" t="inlineStr"/>
+      <c r="J4" s="26" t="inlineStr"/>
+      <c r="K4" s="26" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>LTRP 2025</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr"/>
-      <c r="C5" s="25" t="inlineStr"/>
-      <c r="D5" s="25" t="inlineStr"/>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr"/>
+      <c r="C5" s="26" t="inlineStr"/>
+      <c r="D5" s="26" t="inlineStr"/>
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="26" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="J5" s="25" t="inlineStr">
+      <c r="J5" s="26" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="K5" s="25" t="inlineStr"/>
+      <c r="K5" s="26" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>LTRP 2026</t>
         </is>
       </c>
-      <c r="B6" s="25" t="inlineStr"/>
-      <c r="C6" s="25" t="inlineStr"/>
-      <c r="D6" s="25" t="inlineStr"/>
-      <c r="E6" s="25" t="inlineStr"/>
-      <c r="F6" s="25" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr"/>
+      <c r="C6" s="26" t="inlineStr"/>
+      <c r="D6" s="26" t="inlineStr"/>
+      <c r="E6" s="26" t="inlineStr"/>
+      <c r="F6" s="26" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="G6" s="25" t="inlineStr">
+      <c r="G6" s="26" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="H6" s="25" t="inlineStr">
+      <c r="H6" s="26" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="I6" s="25" t="inlineStr">
+      <c r="I6" s="26" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="J6" s="25" t="inlineStr">
+      <c r="J6" s="26" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="K6" s="25" t="inlineStr">
+      <c r="K6" s="26" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t># planes</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n">
+      <c r="B7" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="26" t="n">
+      <c r="C7" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="D7" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="26" t="n">
+      <c r="G7" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="26" t="n">
+      <c r="H7" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="I7" s="26" t="n">
+      <c r="I7" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="26" t="n">
+      <c r="J7" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="K7" s="26" t="n">
+      <c r="K7" s="27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1879,7 +1905,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>Detalle ene-2027 — base 50/50 × precio acción</t>
         </is>
@@ -2086,19 +2112,19 @@
         <v/>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="28">
+      <c r="D10" s="29">
         <f>SUM(D5:D9)</f>
         <v/>
       </c>
-      <c r="E10" s="28">
+      <c r="E10" s="29">
         <f>SUM(E5:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="28">
+      <c r="F10" s="29">
         <f>SUM(F5:F9)</f>
         <v/>
       </c>
-      <c r="G10" s="28">
+      <c r="G10" s="29">
         <f>SUM(G5:G9)</f>
         <v/>
       </c>
@@ -2114,7 +2140,7 @@
           <t>Base sin acción (factor 1,0)</t>
         </is>
       </c>
-      <c r="B12" s="29" t="n">
+      <c r="B12" s="30" t="n">
         <v>32803.67</v>
       </c>
     </row>
@@ -2124,7 +2150,7 @@
           <t>Estimado con acción (simulación)</t>
         </is>
       </c>
-      <c r="B13" s="29" t="n">
+      <c r="B13" s="30" t="n">
         <v>35332</v>
       </c>
     </row>
@@ -2134,7 +2160,7 @@
           <t>Diferencia = efecto valor de la acción</t>
         </is>
       </c>
-      <c r="B14" s="29" t="n">
+      <c r="B14" s="30" t="n">
         <v>2528.330000000002</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Extend LTRP simulation with Sol age and projected 2027–2036 grants.
Add Edad Sol, assume future 70k plans at flat 11,666 per tranche, and stretch the payment matrix through 2037 while keeping 2026 fully collected only in 2032.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LTRP/LTRP.xlsx
+++ b/LTRP/LTRP.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Simulación de pagos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Planes vigentes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Planes" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Acción estimada" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Calendario vesting" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Detalle fórmula 2027" sheetId="6" state="visible" r:id="rId6"/>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,10 @@
     <font>
       <i val="1"/>
       <color rgb="00595959"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
     </font>
     <font>
       <b val="1"/>
@@ -61,7 +65,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -71,6 +75,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -86,11 +100,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DEEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -120,57 +129,65 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="7" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -537,11 +554,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="91" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="77" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -589,8 +606,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr"/>
-      <c r="B5" s="3" t="inlineStr"/>
+      <c r="A5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -612,165 +629,201 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Otorgado 70.000 en 2026 → ene-2027 = 1/6·2026 + 1/6·2025 + 1/6·2024 + 1/6·2023 + 1/6·2022</t>
+          <t>Otorgado 70.000 en 2026 (edad 45) → ene-2027 = 1/6·2026+…+1/6·2022</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Plan 2026 completo</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Recién en 2032 se cobra el 6/6 y se completa la totalidad del plan otorgado en 2026</t>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Recién en 2032 se cobra el 6/6 y se completa la totalidad del plan</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>Proyección</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>LTRP 2027–2036 asumidos a 70.000 · 1/6≈11.666 sin precio de acción aún</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>Fórmula con acción</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>(N/6)×50% fijo + (N/6)×50% × (P_año / P_otorgamiento)</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr"/>
-      <c r="B10" s="3" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Total estimado a cobrar 2027</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>35332</v>
-      </c>
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Total estimado a cobrar 2028</t>
+          <t>Total estimado 2027 (vigentes)</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>36847</v>
+        <v>35332</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Total estimado a cobrar 2029</t>
+          <t>Total estimado 2028 (con proy. 2027)</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>32284</v>
+        <v>48513</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Total estimado a cobrar 2030</t>
+          <t>Total estimado 2029</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>25001</v>
+        <v>55616</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Total estimado a cobrar 2031</t>
+          <t>Total estimado 2030</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>19379</v>
+        <v>59999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Total estimado a cobrar 2032</t>
+          <t>Total estimado 2031</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>13056</v>
+        <v>66043</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Total acumulado pendiente de pago</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>161899</v>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Total estimado 2032 (cierra plan 2026)</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>71386</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="3" t="inlineStr"/>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Total estimado 2033–2037 (c/u, tope 6×11666)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>69996</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Base 2027 sin efecto acción (suma 1/6)</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="n">
-        <v>32803.67</v>
-      </c>
+      <c r="A19" s="4" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Diferencia 2027 por valor de la acción</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="n">
-        <v>2528.33</v>
+          <t>Pendiente vigentes 2022–2026 (con acción)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>161899</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Precio acción estimado 2027</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="n">
-        <v>1765.02</v>
+          <t>Pendiente total con proyección 2027–2037</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>686869</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr"/>
-      <c r="B22" s="3" t="inlineStr"/>
+      <c r="B22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Metodología precio</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Año 1: promedio 60 días + 3% cierre 2026 · Luego +8% anual</t>
-        </is>
+          <t>Base 2027 sin efecto acción</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>32803.67</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t>Diferencia 2027 por valor de la acción</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>2528.33</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Precio acción estimado 2027</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>1765.02</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Edad Sol</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Columna por plan al año de otorgamiento (41 en LTRP 2022 … 51 en LTRP 2036)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Ingreso por bono MELI; independiente de CIUDAD / SOL / propiedades.</t>
         </is>
@@ -787,18 +840,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -811,316 +871,856 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Última actualización: agosto 2026 · Máx. 6 planes · cada enero = suma de 1/6 ajustados por acción MELI</t>
-        </is>
+          <t>Máx. 6 planes por enero · 50% fijo + 50% variable (acción MELI) · Planes 2027+ proyectados a 70.000 con 1/6≈11.666 (sin precio de acción aún) · Plan 2026 se completa recién en 2032</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="F3" s="10" t="n">
+        <v>2027</v>
+      </c>
+      <c r="G3" s="10" t="n">
+        <v>2028</v>
+      </c>
+      <c r="H3" s="10" t="n">
+        <v>2029</v>
+      </c>
+      <c r="I3" s="10" t="n">
+        <v>2030</v>
+      </c>
+      <c r="J3" s="10" t="n">
+        <v>2031</v>
+      </c>
+      <c r="K3" s="10" t="n">
+        <v>2032</v>
+      </c>
+      <c r="L3" s="10" t="n">
+        <v>2033</v>
+      </c>
+      <c r="M3" s="10" t="n">
+        <v>2034</v>
+      </c>
+      <c r="N3" s="10" t="n">
+        <v>2035</v>
+      </c>
+      <c r="O3" s="10" t="n">
+        <v>2036</v>
+      </c>
+      <c r="P3" s="10" t="n">
+        <v>2037</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Edad Sol</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Valor nominal</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Valor por año Aprox</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Valor de acción al otorgamiento</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>2028</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>2029</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>2030</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>2031</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2032</t>
         </is>
       </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>2033</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>2034</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>2035</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>2036</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>2037</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="11" t="n">
+        <v>41</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>LTRP 2022</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="C5" s="6" t="n">
         <v>30000</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="D5" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E5" s="7" t="n">
         <v>1391.81</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="F5" s="12" t="n">
         <v>5670</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="G5" s="13" t="n">
         <v>5924</v>
       </c>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="n"/>
+      <c r="N5" s="3" t="n"/>
+      <c r="O5" s="3" t="n"/>
+      <c r="P5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="11" t="n">
+        <v>42</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>LTRP 2023</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="C6" s="6" t="n">
         <v>30000</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="D6" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E6" s="7" t="n">
         <v>888.6900000000001</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="F6" s="12" t="n">
         <v>7465</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="G6" s="13" t="n">
         <v>7862</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="H6" s="13" t="n">
         <v>8291</v>
       </c>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
+      <c r="N6" s="3" t="n"/>
+      <c r="O6" s="3" t="n"/>
+      <c r="P6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="11" t="n">
+        <v>43</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>LTRP 2024</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="C7" s="6" t="n">
         <v>30000</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="D7" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E7" s="7" t="n">
         <v>1426.11</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="F7" s="12" t="n">
         <v>5594</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="G7" s="13" t="n">
         <v>5842</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="H7" s="13" t="n">
         <v>6109</v>
       </c>
-      <c r="G7" s="11" t="n">
+      <c r="I7" s="13" t="n">
         <v>6398</v>
       </c>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
+      <c r="N7" s="3" t="n"/>
+      <c r="O7" s="3" t="n"/>
+      <c r="P7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="11" t="n">
+        <v>44</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>LTRP 2025</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="C8" s="6" t="n">
         <v>36822</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="D8" s="7" t="n">
+        <v>6137</v>
+      </c>
+      <c r="E8" s="7" t="n">
         <v>1944.47</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="F8" s="12" t="n">
         <v>5854</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="G8" s="13" t="n">
         <v>6077</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="H8" s="13" t="n">
         <v>6317</v>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="I8" s="13" t="n">
         <v>6577</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="J8" s="13" t="n">
         <v>6858</v>
       </c>
-      <c r="I8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="3" t="n"/>
+      <c r="N8" s="3" t="n"/>
+      <c r="O8" s="3" t="n"/>
+      <c r="P8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>LTRP 2026</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="C9" s="6" t="n">
         <v>70000</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="D9" s="7" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="E9" s="7" t="n">
         <v>2094.65</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="F9" s="12" t="n">
         <v>10749</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="G9" s="13" t="n">
         <v>11142</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="H9" s="13" t="n">
         <v>11567</v>
       </c>
-      <c r="G9" s="11" t="n">
+      <c r="I9" s="13" t="n">
         <v>12026</v>
       </c>
-      <c r="H9" s="11" t="n">
+      <c r="J9" s="13" t="n">
         <v>12521</v>
       </c>
-      <c r="I9" s="11" t="n">
+      <c r="K9" s="13" t="n">
         <v>13056</v>
       </c>
+      <c r="L9" s="3" t="n"/>
+      <c r="M9" s="3" t="n"/>
+      <c r="N9" s="3" t="n"/>
+      <c r="O9" s="3" t="n"/>
+      <c r="P9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2027</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="H10" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="I10" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="J10" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="K10" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="L10" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="M10" s="3" t="n"/>
+      <c r="N10" s="3" t="n"/>
+      <c r="O10" s="3" t="n"/>
+      <c r="P10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>47</v>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2028</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="I11" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="J11" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="K11" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="L11" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="M11" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="N11" s="3" t="n"/>
+      <c r="O11" s="3" t="n"/>
+      <c r="P11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
+        <v>47</v>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2029</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="J12" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="K12" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="L12" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="M12" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="N12" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="O12" s="3" t="n"/>
+      <c r="P12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="n">
+        <v>48</v>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2030</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="K13" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="L13" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="M13" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="N13" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="O13" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="P13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="n">
+        <v>48</v>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2031</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="n"/>
+      <c r="K14" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="L14" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="M14" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="N14" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="O14" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="P14" s="18" t="n">
+        <v>11666</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="n">
+        <v>49</v>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2032</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="M15" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="N15" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="O15" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="P15" s="18" t="n">
+        <v>11666</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="n">
+        <v>49</v>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2033</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="3" t="n"/>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="n"/>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="N16" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="O16" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="P16" s="18" t="n">
+        <v>11666</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2034</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D17" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="n"/>
+      <c r="N17" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="O17" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="P17" s="18" t="n">
+        <v>11666</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2035</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D18" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="3" t="n"/>
+      <c r="N18" s="3" t="n"/>
+      <c r="O18" s="18" t="n">
+        <v>11666</v>
+      </c>
+      <c r="P18" s="18" t="n">
+        <v>11666</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="n">
+        <v>51</v>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2036</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D19" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
+      <c r="J19" s="3" t="n"/>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="n"/>
+      <c r="M19" s="3" t="n"/>
+      <c r="N19" s="3" t="n"/>
+      <c r="O19" s="3" t="n"/>
+      <c r="P19" s="18" t="n">
+        <v>11666</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr"/>
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Total estimado a cobrar por año</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n"/>
-      <c r="C10" s="13" t="n"/>
-      <c r="D10" s="14">
-        <f>SUM(D5:D9)</f>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="20">
+        <f>SUM(F5:F19)</f>
         <v/>
       </c>
-      <c r="E10" s="14">
-        <f>SUM(E5:E9)</f>
+      <c r="G20" s="20">
+        <f>SUM(G5:G19)</f>
         <v/>
       </c>
-      <c r="F10" s="14">
-        <f>SUM(F5:F9)</f>
+      <c r="H20" s="20">
+        <f>SUM(H5:H19)</f>
         <v/>
       </c>
-      <c r="G10" s="14">
-        <f>SUM(G5:G9)</f>
+      <c r="I20" s="20">
+        <f>SUM(I5:I19)</f>
         <v/>
       </c>
-      <c r="H10" s="14">
-        <f>SUM(H5:H9)</f>
+      <c r="J20" s="20">
+        <f>SUM(J5:J19)</f>
         <v/>
       </c>
-      <c r="I10" s="14">
-        <f>SUM(I5:I9)</f>
+      <c r="K20" s="20">
+        <f>SUM(K5:K19)</f>
         <v/>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="L20" s="20">
+        <f>SUM(L5:L19)</f>
+        <v/>
+      </c>
+      <c r="M20" s="20">
+        <f>SUM(M5:M19)</f>
+        <v/>
+      </c>
+      <c r="N20" s="20">
+        <f>SUM(N5:N19)</f>
+        <v/>
+      </c>
+      <c r="O20" s="20">
+        <f>SUM(O5:O19)</f>
+        <v/>
+      </c>
+      <c r="P20" s="20">
+        <f>SUM(P5:P19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>Valor de la acción estimado</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>El valor de acción considerado para el primer año corresponde al promedio de los últimos 60 días de trading al momento de actualizar esta simulación con un ajuste de 3% correspondiente al cierre del 2026. Para los años subsiguientes se considera un crecimiento anual del 8%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+    <row r="23" ht="40" customHeight="1">
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Año 1 (2027): promedio últimos 60 días de trading + ajuste 3% cierre 2026. Años siguientes: crecimiento anual 8%. Planes 2027+ aún sin precio al otorgamiento → placeholder 11.666 (1/6 nominal).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="23" t="inlineStr">
         <is>
           <t>Precio estimado</t>
         </is>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="F24" s="24" t="n">
         <v>1765.02</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="G24" s="24" t="n">
         <v>1906.22</v>
       </c>
-      <c r="F14" s="18" t="n">
+      <c r="H24" s="24" t="n">
         <v>2058.72</v>
       </c>
-      <c r="G14" s="18" t="n">
+      <c r="I24" s="24" t="n">
         <v>2223.42</v>
       </c>
-      <c r="H14" s="18" t="n">
+      <c r="J24" s="24" t="n">
         <v>2401.29</v>
       </c>
-      <c r="I14" s="18" t="n">
+      <c r="K24" s="24" t="n">
         <v>2593.39</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Total acumulado pendiente de pago</t>
-        </is>
-      </c>
-      <c r="B16" s="19">
-        <f>SUM(D10:I10)</f>
+      <c r="L24" s="14" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M24" s="14" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="N24" s="14" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="O24" s="14" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="P24" s="14" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>Total acumulado pendiente de pago (con proyección)</t>
+        </is>
+      </c>
+      <c r="C26" s="25">
+        <f>SUM(F20:P20)</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Fórmula por celda</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>ROUND( (Nominal÷6)×50% + (Nominal÷6)×50% × (P_año / P_otorgamiento) ; 0 )</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Pendiente planes vigentes 2022–2026 (simulación con acción)</t>
+        </is>
+      </c>
+      <c r="C27" s="26" t="n">
+        <v>161899</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>Fórmula (planes con precio al otorgamiento)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ROUND( (N÷6)×50% + (N÷6)×50% × (P_año / P_otorgamiento) ; 0 )</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1">
+      <c r="B30" s="23" t="inlineStr">
         <is>
           <t>Regla general</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>Máximo 6 planes. Cada enero se suma el 1/6 de cada plan activo. Ej.: otorgado 70.000 en 2026 → ene-2027 = 1/6·2026 + 1/6·2025 + … + 1/6·2022, cada tramo ajustado 50/50 por la acción. Recién en 2032 se cobra el 6/6 y se completa la totalidad del plan 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="17" t="inlineStr">
-        <is>
-          <t>Plan LTRP 2026 (70.000)</t>
-        </is>
-      </c>
-      <c r="B21" s="20" t="inlineStr">
-        <is>
-          <t>6 cobros ene-2027…ene-2032 · la totalidad del plan se completa recién en 2032 (último 1/6 = 13.056)</t>
+      <c r="C30" s="22" t="inlineStr">
+        <is>
+          <t>Máximo 6 planes por cobro de enero. Ej.: otorgado 70.000 en 2026 → ene-2027 = 1/6·2026+…+1/6·2022. Recién en 2032 se completa la totalidad del plan 2026. Filas grises = proyección futura (nominal 70.000 asumido).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="B23:P23"/>
+    <mergeCell ref="C30:P30"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1132,268 +1732,520 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="33" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>Edad Sol</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Año grant</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Valor nominal</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Valor por año Aprox</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Valor de acción al otorgamiento</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>1/6 anual (base)</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Fijo 50% base</t>
-        </is>
-      </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Variable 50% base</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
           <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>LTRP 2022</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="C2" s="3" t="n">
         <v>2022</v>
       </c>
-      <c r="C2" s="6" t="n">
+      <c r="D2" s="6" t="n">
         <v>30000</v>
-      </c>
-      <c r="D2" s="7" t="n">
-        <v>1391.81</v>
       </c>
       <c r="E2" s="7" t="n">
         <v>5000</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G2" s="7" t="n">
-        <v>2500</v>
+        <v>1391.81</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>vigente</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>Últimos cobros ene-2027 y ene-2028</t>
+          <t>Últimos cobros 2027-2028</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>LTRP 2023</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="C3" s="3" t="n">
         <v>2023</v>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="D3" s="6" t="n">
         <v>30000</v>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>888.6900000000001</v>
       </c>
       <c r="E3" s="7" t="n">
         <v>5000</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G3" s="7" t="n">
-        <v>2500</v>
+        <v>888.6900000000001</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>vigente</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Cobros ene-2027 a ene-2029</t>
+          <t>Cobros 2027-2029</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>LTRP 2024</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="C4" s="3" t="n">
         <v>2024</v>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="D4" s="6" t="n">
         <v>30000</v>
-      </c>
-      <c r="D4" s="7" t="n">
-        <v>1426.11</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>5000</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G4" s="7" t="n">
-        <v>2500</v>
+        <v>1426.11</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>vigente</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Cobros ene-2027 a ene-2030</t>
+          <t>Cobros 2027-2030</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>LTRP 2025</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="C5" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="D5" s="6" t="n">
         <v>36822</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>1944.47</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>6137</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>3068.5</v>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>3068.5</v>
+        <v>1944.47</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
+          <t>Cobros 2027-2031</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>LTRP 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>2094.65</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
           <t>vigente</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Cobros ene-2027 a ene-2031</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>LTRP 2026</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C6" s="6" t="n">
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Cobros 2027-2032 · completo recién en 2032</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="n">
+        <v>46</v>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2027</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D7" s="16" t="n">
         <v>70000</v>
       </c>
-      <c r="D6" s="7" t="n">
-        <v>2094.65</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>11666.66666666667</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>5833.333333333333</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>5833.333333333333</v>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>vigente</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>6 cobros ene-2027…ene-2032 · recién en 2032 se completa la totalidad del plan otorgado en 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="22">
-        <f>SUM(C2:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="23">
-        <f>SUM(E2:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="23">
-        <f>SUM(F2:F6)</f>
-        <v/>
-      </c>
-      <c r="G7" s="23">
-        <f>SUM(G2:G6)</f>
-        <v/>
-      </c>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
+      <c r="E7" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="F7" s="15" t="n"/>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>proyectado</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>Placeholder 1/6≈11666 sin precio de acción aún · cobros 2028-2033</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="n">
+        <v>47</v>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2028</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="F8" s="15" t="n"/>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>proyectado</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Placeholder · cobros 2029-2034</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="n">
+        <v>47</v>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2029</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="F9" s="15" t="n"/>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>proyectado</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>Placeholder · cobros 2030-2035</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="n">
+        <v>48</v>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2030</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>2030</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>proyectado</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Placeholder · cobros 2031-2036</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="n">
+        <v>48</v>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2031</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>2031</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>proyectado</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>Placeholder · cobros 2032-2037</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="n">
+        <v>49</v>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2032</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>2032</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>proyectado</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>Placeholder · cobros 2033-2038 (parcial en matriz hasta 2037)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="n">
+        <v>49</v>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2033</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>2033</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>proyectado</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>Placeholder · cobros 2034-2039 (parcial hasta 2037)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2034</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>2034</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="F14" s="15" t="n"/>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>proyectado</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>Placeholder · cobros 2035-2040 (parcial hasta 2037)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2035</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>2035</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="F15" s="15" t="n"/>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>proyectado</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="inlineStr">
+        <is>
+          <t>Placeholder · cobros 2036-2041 (parcial hasta 2037)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="n">
+        <v>51</v>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>LTRP 2036</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>2036</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>11666.67</v>
+      </c>
+      <c r="F16" s="15" t="n"/>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>proyectado</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>Placeholder · primer cobro 2037</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1410,7 +2262,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="61" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1435,7 +2287,7 @@
       <c r="A2" s="3" t="n">
         <v>2027</v>
       </c>
-      <c r="B2" s="24" t="n">
+      <c r="B2" s="27" t="n">
         <v>1765.02</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -1448,7 +2300,7 @@
       <c r="A3" s="3" t="n">
         <v>2028</v>
       </c>
-      <c r="B3" s="24" t="n">
+      <c r="B3" s="27" t="n">
         <v>1906.22</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1461,7 +2313,7 @@
       <c r="A4" s="3" t="n">
         <v>2029</v>
       </c>
-      <c r="B4" s="24" t="n">
+      <c r="B4" s="27" t="n">
         <v>2058.72</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1474,7 +2326,7 @@
       <c r="A5" s="3" t="n">
         <v>2030</v>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="27" t="n">
         <v>2223.42</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1487,7 +2339,7 @@
       <c r="A6" s="3" t="n">
         <v>2031</v>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="27" t="n">
         <v>2401.29</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1500,7 +2352,7 @@
       <c r="A7" s="3" t="n">
         <v>2032</v>
       </c>
-      <c r="B7" s="24" t="n">
+      <c r="B7" s="27" t="n">
         <v>2593.39</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1511,7 +2363,7 @@
     </row>
     <row r="8"/>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>Metodología</t>
         </is>
@@ -1526,7 +2378,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Promedio últimos 60 días de trading + ajuste 3% cierre 2026</t>
+          <t>Promedio 60 días trading + ajuste 3% cierre 2026</t>
         </is>
       </c>
     </row>
@@ -1545,12 +2397,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fórmula pago</t>
+          <t>Planes 2027+</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ROUND((N/6)*50% + (N/6)*50%*(P_año/P_otorgamiento); 0)</t>
+          <t>Sin precio al otorgamiento aún → simulación usa 11.666 (1/6 de 70.000)</t>
         </is>
       </c>
     </row>
@@ -1565,319 +2417,789 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>Plan</t>
         </is>
       </c>
-      <c r="B1" s="25" t="inlineStr">
+      <c r="B1" s="28" t="inlineStr">
         <is>
           <t>31/01/2023</t>
         </is>
       </c>
-      <c r="C1" s="25" t="inlineStr">
+      <c r="C1" s="28" t="inlineStr">
         <is>
           <t>31/01/2024</t>
         </is>
       </c>
-      <c r="D1" s="25" t="inlineStr">
+      <c r="D1" s="28" t="inlineStr">
         <is>
           <t>31/01/2025</t>
         </is>
       </c>
-      <c r="E1" s="25" t="inlineStr">
+      <c r="E1" s="28" t="inlineStr">
         <is>
           <t>31/01/2026</t>
         </is>
       </c>
-      <c r="F1" s="25" t="inlineStr">
+      <c r="F1" s="28" t="inlineStr">
         <is>
           <t>31/01/2027</t>
         </is>
       </c>
-      <c r="G1" s="25" t="inlineStr">
+      <c r="G1" s="28" t="inlineStr">
         <is>
           <t>31/01/2028</t>
         </is>
       </c>
-      <c r="H1" s="25" t="inlineStr">
+      <c r="H1" s="28" t="inlineStr">
         <is>
           <t>31/01/2029</t>
         </is>
       </c>
-      <c r="I1" s="25" t="inlineStr">
+      <c r="I1" s="28" t="inlineStr">
         <is>
           <t>31/01/2030</t>
         </is>
       </c>
-      <c r="J1" s="25" t="inlineStr">
+      <c r="J1" s="28" t="inlineStr">
         <is>
           <t>31/01/2031</t>
         </is>
       </c>
-      <c r="K1" s="25" t="inlineStr">
+      <c r="K1" s="28" t="inlineStr">
         <is>
           <t>31/01/2032</t>
         </is>
       </c>
+      <c r="L1" s="28" t="inlineStr">
+        <is>
+          <t>31/01/2033</t>
+        </is>
+      </c>
+      <c r="M1" s="28" t="inlineStr">
+        <is>
+          <t>31/01/2034</t>
+        </is>
+      </c>
+      <c r="N1" s="28" t="inlineStr">
+        <is>
+          <t>31/01/2035</t>
+        </is>
+      </c>
+      <c r="O1" s="28" t="inlineStr">
+        <is>
+          <t>31/01/2036</t>
+        </is>
+      </c>
+      <c r="P1" s="28" t="inlineStr">
+        <is>
+          <t>31/01/2037</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>LTRP 2022</t>
         </is>
       </c>
-      <c r="B2" s="26" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="C2" s="26" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="D2" s="26" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="E2" s="26" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="F2" s="26" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="G2" s="26" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="H2" s="26" t="inlineStr"/>
-      <c r="I2" s="26" t="inlineStr"/>
-      <c r="J2" s="26" t="inlineStr"/>
-      <c r="K2" s="26" t="inlineStr"/>
+      <c r="H2" s="11" t="inlineStr"/>
+      <c r="I2" s="11" t="inlineStr"/>
+      <c r="J2" s="11" t="inlineStr"/>
+      <c r="K2" s="11" t="inlineStr"/>
+      <c r="L2" s="11" t="inlineStr"/>
+      <c r="M2" s="11" t="inlineStr"/>
+      <c r="N2" s="11" t="inlineStr"/>
+      <c r="O2" s="11" t="inlineStr"/>
+      <c r="P2" s="11" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="26" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>LTRP 2023</t>
         </is>
       </c>
-      <c r="B3" s="26" t="inlineStr"/>
-      <c r="C3" s="26" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr"/>
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="D3" s="26" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="E3" s="26" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="F3" s="26" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="G3" s="26" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="H3" s="26" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="I3" s="26" t="inlineStr"/>
-      <c r="J3" s="26" t="inlineStr"/>
-      <c r="K3" s="26" t="inlineStr"/>
+      <c r="I3" s="11" t="inlineStr"/>
+      <c r="J3" s="11" t="inlineStr"/>
+      <c r="K3" s="11" t="inlineStr"/>
+      <c r="L3" s="11" t="inlineStr"/>
+      <c r="M3" s="11" t="inlineStr"/>
+      <c r="N3" s="11" t="inlineStr"/>
+      <c r="O3" s="11" t="inlineStr"/>
+      <c r="P3" s="11" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>LTRP 2024</t>
         </is>
       </c>
-      <c r="B4" s="26" t="inlineStr"/>
-      <c r="C4" s="26" t="inlineStr"/>
-      <c r="D4" s="26" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr"/>
+      <c r="C4" s="11" t="inlineStr"/>
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="E4" s="26" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="F4" s="26" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="G4" s="26" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="H4" s="26" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="I4" s="26" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="J4" s="26" t="inlineStr"/>
-      <c r="K4" s="26" t="inlineStr"/>
+      <c r="J4" s="11" t="inlineStr"/>
+      <c r="K4" s="11" t="inlineStr"/>
+      <c r="L4" s="11" t="inlineStr"/>
+      <c r="M4" s="11" t="inlineStr"/>
+      <c r="N4" s="11" t="inlineStr"/>
+      <c r="O4" s="11" t="inlineStr"/>
+      <c r="P4" s="11" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>LTRP 2025</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr"/>
-      <c r="C5" s="26" t="inlineStr"/>
-      <c r="D5" s="26" t="inlineStr"/>
-      <c r="E5" s="26" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr"/>
+      <c r="C5" s="11" t="inlineStr"/>
+      <c r="D5" s="11" t="inlineStr"/>
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="F5" s="26" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="G5" s="26" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="H5" s="26" t="inlineStr">
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="I5" s="26" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="J5" s="26" t="inlineStr">
+      <c r="J5" s="11" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="K5" s="26" t="inlineStr"/>
+      <c r="K5" s="11" t="inlineStr"/>
+      <c r="L5" s="11" t="inlineStr"/>
+      <c r="M5" s="11" t="inlineStr"/>
+      <c r="N5" s="11" t="inlineStr"/>
+      <c r="O5" s="11" t="inlineStr"/>
+      <c r="P5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>LTRP 2026</t>
         </is>
       </c>
-      <c r="B6" s="26" t="inlineStr"/>
-      <c r="C6" s="26" t="inlineStr"/>
-      <c r="D6" s="26" t="inlineStr"/>
-      <c r="E6" s="26" t="inlineStr"/>
-      <c r="F6" s="26" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr"/>
+      <c r="C6" s="11" t="inlineStr"/>
+      <c r="D6" s="11" t="inlineStr"/>
+      <c r="E6" s="11" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="G6" s="26" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="H6" s="26" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="I6" s="26" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="J6" s="26" t="inlineStr">
+      <c r="J6" s="11" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="K6" s="26" t="inlineStr">
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
+      <c r="L6" s="11" t="inlineStr"/>
+      <c r="M6" s="11" t="inlineStr"/>
+      <c r="N6" s="11" t="inlineStr"/>
+      <c r="O6" s="11" t="inlineStr"/>
+      <c r="P6" s="11" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>LTRP 2027</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr"/>
+      <c r="C7" s="11" t="inlineStr"/>
+      <c r="D7" s="11" t="inlineStr"/>
+      <c r="E7" s="11" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr"/>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>1/6</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="M7" s="11" t="inlineStr"/>
+      <c r="N7" s="11" t="inlineStr"/>
+      <c r="O7" s="11" t="inlineStr"/>
+      <c r="P7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>LTRP 2028</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr"/>
+      <c r="C8" s="11" t="inlineStr"/>
+      <c r="D8" s="11" t="inlineStr"/>
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="11" t="inlineStr"/>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>1/6</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="L8" s="11" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="M8" s="11" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="N8" s="11" t="inlineStr"/>
+      <c r="O8" s="11" t="inlineStr"/>
+      <c r="P8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>LTRP 2029</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr"/>
+      <c r="C9" s="11" t="inlineStr"/>
+      <c r="D9" s="11" t="inlineStr"/>
+      <c r="E9" s="11" t="inlineStr"/>
+      <c r="F9" s="11" t="inlineStr"/>
+      <c r="G9" s="11" t="inlineStr"/>
+      <c r="H9" s="11" t="inlineStr"/>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>1/6</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="M9" s="11" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="N9" s="11" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="O9" s="11" t="inlineStr"/>
+      <c r="P9" s="11" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>LTRP 2030</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr"/>
+      <c r="C10" s="11" t="inlineStr"/>
+      <c r="D10" s="11" t="inlineStr"/>
+      <c r="E10" s="11" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr"/>
+      <c r="G10" s="11" t="inlineStr"/>
+      <c r="H10" s="11" t="inlineStr"/>
+      <c r="I10" s="11" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>1/6</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="L10" s="11" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="M10" s="11" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="N10" s="11" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="O10" s="11" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="P10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>LTRP 2031</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr"/>
+      <c r="C11" s="11" t="inlineStr"/>
+      <c r="D11" s="11" t="inlineStr"/>
+      <c r="E11" s="11" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr"/>
+      <c r="G11" s="11" t="inlineStr"/>
+      <c r="H11" s="11" t="inlineStr"/>
+      <c r="I11" s="11" t="inlineStr"/>
+      <c r="J11" s="11" t="inlineStr"/>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>1/6</t>
+        </is>
+      </c>
+      <c r="L11" s="11" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="M11" s="11" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="N11" s="11" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="O11" s="11" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="P11" s="11" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>LTRP 2032</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr"/>
+      <c r="C12" s="11" t="inlineStr"/>
+      <c r="D12" s="11" t="inlineStr"/>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
+      <c r="G12" s="11" t="inlineStr"/>
+      <c r="H12" s="11" t="inlineStr"/>
+      <c r="I12" s="11" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="11" t="inlineStr"/>
+      <c r="L12" s="11" t="inlineStr">
+        <is>
+          <t>1/6</t>
+        </is>
+      </c>
+      <c r="M12" s="11" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="N12" s="11" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="O12" s="11" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="P12" s="11" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>LTRP 2033</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr"/>
+      <c r="C13" s="11" t="inlineStr"/>
+      <c r="D13" s="11" t="inlineStr"/>
+      <c r="E13" s="11" t="inlineStr"/>
+      <c r="F13" s="11" t="inlineStr"/>
+      <c r="G13" s="11" t="inlineStr"/>
+      <c r="H13" s="11" t="inlineStr"/>
+      <c r="I13" s="11" t="inlineStr"/>
+      <c r="J13" s="11" t="inlineStr"/>
+      <c r="K13" s="11" t="inlineStr"/>
+      <c r="L13" s="11" t="inlineStr"/>
+      <c r="M13" s="11" t="inlineStr">
+        <is>
+          <t>1/6</t>
+        </is>
+      </c>
+      <c r="N13" s="11" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="O13" s="11" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="P13" s="11" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>LTRP 2034</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr"/>
+      <c r="C14" s="11" t="inlineStr"/>
+      <c r="D14" s="11" t="inlineStr"/>
+      <c r="E14" s="11" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
+      <c r="G14" s="11" t="inlineStr"/>
+      <c r="H14" s="11" t="inlineStr"/>
+      <c r="I14" s="11" t="inlineStr"/>
+      <c r="J14" s="11" t="inlineStr"/>
+      <c r="K14" s="11" t="inlineStr"/>
+      <c r="L14" s="11" t="inlineStr"/>
+      <c r="M14" s="11" t="inlineStr"/>
+      <c r="N14" s="11" t="inlineStr">
+        <is>
+          <t>1/6</t>
+        </is>
+      </c>
+      <c r="O14" s="11" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="P14" s="11" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>LTRP 2035</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr"/>
+      <c r="C15" s="11" t="inlineStr"/>
+      <c r="D15" s="11" t="inlineStr"/>
+      <c r="E15" s="11" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr"/>
+      <c r="G15" s="11" t="inlineStr"/>
+      <c r="H15" s="11" t="inlineStr"/>
+      <c r="I15" s="11" t="inlineStr"/>
+      <c r="J15" s="11" t="inlineStr"/>
+      <c r="K15" s="11" t="inlineStr"/>
+      <c r="L15" s="11" t="inlineStr"/>
+      <c r="M15" s="11" t="inlineStr"/>
+      <c r="N15" s="11" t="inlineStr"/>
+      <c r="O15" s="11" t="inlineStr">
+        <is>
+          <t>1/6</t>
+        </is>
+      </c>
+      <c r="P15" s="11" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>LTRP 2036</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr"/>
+      <c r="C16" s="11" t="inlineStr"/>
+      <c r="D16" s="11" t="inlineStr"/>
+      <c r="E16" s="11" t="inlineStr"/>
+      <c r="F16" s="11" t="inlineStr"/>
+      <c r="G16" s="11" t="inlineStr"/>
+      <c r="H16" s="11" t="inlineStr"/>
+      <c r="I16" s="11" t="inlineStr"/>
+      <c r="J16" s="11" t="inlineStr"/>
+      <c r="K16" s="11" t="inlineStr"/>
+      <c r="L16" s="11" t="inlineStr"/>
+      <c r="M16" s="11" t="inlineStr"/>
+      <c r="N16" s="11" t="inlineStr"/>
+      <c r="O16" s="11" t="inlineStr"/>
+      <c r="P16" s="11" t="inlineStr">
+        <is>
+          <t>1/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t># planes</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B17" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C17" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D17" s="29" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E17" s="29" t="n">
         <v>4</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F17" s="29" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="27" t="n">
-        <v>5</v>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>4</v>
-      </c>
-      <c r="I7" s="27" t="n">
-        <v>3</v>
-      </c>
-      <c r="J7" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="K7" s="27" t="n">
-        <v>1</v>
+      <c r="G17" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="I17" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="J17" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="K17" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="L17" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="M17" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="N17" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="O17" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="P17" s="29" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1891,23 +3213,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="28" t="inlineStr">
-        <is>
-          <t>Detalle ene-2027 — base 50/50 × precio acción</t>
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Detalle ene-2027 — solo planes vigentes con precio de acción</t>
         </is>
       </c>
     </row>
@@ -1922,214 +3245,235 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Edad</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
           <t>Plan</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Nominal</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>P otorgamiento</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Fijo 50%</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Variable 50% × (P2027/Pgrant)</t>
-        </is>
-      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>Variable ajustada</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>Total (sin round)</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Total simulación (round)</t>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Simulación (round)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>LTRP 2022</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="C5" s="6" t="n">
         <v>30000</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="D5" s="7" t="n">
         <v>1391.81</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="E5" s="7" t="n">
         <v>5000</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="F5" s="7" t="n">
         <v>2500</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="G5" s="7" t="n">
         <v>3170.368081850253</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="H5" s="7" t="n">
         <v>5670.368081850253</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="I5" s="6" t="n">
         <v>5670</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>LTRP 2023</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="C6" s="6" t="n">
         <v>30000</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="D6" s="7" t="n">
         <v>888.6900000000001</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="E6" s="7" t="n">
         <v>5000</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="F6" s="7" t="n">
         <v>2500</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="G6" s="7" t="n">
         <v>4965.229720149883</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="H6" s="7" t="n">
         <v>7465.229720149883</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="I6" s="6" t="n">
         <v>7465</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>LTRP 2024</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="C7" s="6" t="n">
         <v>30000</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="D7" s="7" t="n">
         <v>1426.11</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="E7" s="7" t="n">
         <v>5000</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="F7" s="7" t="n">
         <v>2500</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="G7" s="7" t="n">
         <v>3094.11616214738</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="H7" s="7" t="n">
         <v>5594.11616214738</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="I7" s="6" t="n">
         <v>5594</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>LTRP 2025</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="C8" s="6" t="n">
         <v>36822</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="D8" s="7" t="n">
         <v>1944.47</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="E8" s="7" t="n">
         <v>6137</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="F8" s="7" t="n">
         <v>3068.5</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="G8" s="7" t="n">
         <v>2785.316240415126</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="H8" s="7" t="n">
         <v>5853.816240415126</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="I8" s="6" t="n">
         <v>5854</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>LTRP 2026</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="C9" s="6" t="n">
         <v>70000</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="D9" s="7" t="n">
         <v>2094.65</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="E9" s="7" t="n">
         <v>11666.66666666667</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="F9" s="7" t="n">
         <v>5833.333333333333</v>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="G9" s="7" t="n">
         <v>4915.355787363043</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="H9" s="7" t="n">
         <v>10748.68912069638</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="I9" s="6" t="n">
         <v>10749</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B10" s="5">
-        <f>SUM(B5:B9)</f>
+      <c r="C10" s="5">
+        <f>SUM(C5:C9)</f>
         <v/>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="29">
-        <f>SUM(D5:D9)</f>
-        <v/>
-      </c>
-      <c r="E10" s="29">
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="31">
         <f>SUM(E5:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="29">
+      <c r="F10" s="31">
         <f>SUM(F5:F9)</f>
         <v/>
       </c>
-      <c r="G10" s="29">
+      <c r="G10" s="31">
         <f>SUM(G5:G9)</f>
         <v/>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="31">
         <f>SUM(H5:H9)</f>
+        <v/>
+      </c>
+      <c r="I10" s="5">
+        <f>SUM(I5:I9)</f>
         <v/>
       </c>
     </row>
@@ -2137,20 +3481,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Base sin acción (factor 1,0)</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="n">
+          <t>Base sin acción (suma 1/6)</t>
+        </is>
+      </c>
+      <c r="B12" s="32" t="n">
         <v>32803.67</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Estimado con acción (simulación)</t>
-        </is>
-      </c>
-      <c r="B13" s="30" t="n">
+          <t>Estimado con acción</t>
+        </is>
+      </c>
+      <c r="B13" s="32" t="n">
         <v>35332</v>
       </c>
     </row>
@@ -2160,8 +3504,8 @@
           <t>Diferencia = efecto valor de la acción</t>
         </is>
       </c>
-      <c r="B14" s="30" t="n">
-        <v>2528.330000000002</v>
+      <c r="B14" s="32" t="n">
+        <v>2528.33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>